<commit_message>
N3: text pipes only where wording names an earlier pick
</commit_message>
<xml_diff>
--- a/out/C01_chronic_care_patient_journey/agent3/agent3_test_cases_for_review.xlsx
+++ b/out/C01_chronic_care_patient_journey/agent3/agent3_test_cases_for_review.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K161"/>
+  <dimension ref="A1:K160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -9525,12 +9525,12 @@
       </c>
       <c r="E129" s="2" t="inlineStr">
         <is>
-          <t>TC-42363fd1b9</t>
+          <t>TC-524d7f1984</t>
         </is>
       </c>
       <c r="F129" s="3" t="inlineStr">
         <is>
-          <t>Q21's wording comes from Q19's answer: the earlier answer should appear in the wording</t>
+          <t>Prove Q21 REJECTS an answer that breaks its rule. The QRE's rule is: the answer must be at least 5 characters; the answer must be at most 500 characters</t>
         </is>
       </c>
       <c r="G129" s="3" t="inlineStr">
@@ -9561,17 +9561,17 @@
       </c>
       <c r="H129" s="3" t="inlineStr">
         <is>
-          <t>At Q21, type “xxxxx”, then submit.</t>
+          <t>At Q21, type a 500-character answer, then submit.</t>
         </is>
       </c>
       <c r="I129" s="3" t="inlineStr">
         <is>
-          <t>1. Q21's wording includes the words: Concept A</t>
+          <t>1. the survey ACCEPTS the answer and moves to the next page</t>
         </is>
       </c>
       <c r="J129" s="2" t="inlineStr">
         <is>
-          <t>Wording carried forward</t>
+          <t>Answer rule accepts or rejects</t>
         </is>
       </c>
       <c r="K129" s="2" t="inlineStr">
@@ -9601,7 +9601,7 @@
       </c>
       <c r="E130" s="2" t="inlineStr">
         <is>
-          <t>TC-524d7f1984</t>
+          <t>TC-8aaf18bb07</t>
         </is>
       </c>
       <c r="F130" s="3" t="inlineStr">
@@ -9637,7 +9637,7 @@
       </c>
       <c r="H130" s="3" t="inlineStr">
         <is>
-          <t>At Q21, type a 500-character answer, then submit.</t>
+          <t>At Q21, type “O'Brien said "yes" &lt;50% &amp; more”, then submit.</t>
         </is>
       </c>
       <c r="I130" s="3" t="inlineStr">
@@ -9677,12 +9677,12 @@
       </c>
       <c r="E131" s="2" t="inlineStr">
         <is>
-          <t>TC-8aaf18bb07</t>
+          <t>TC-2b316ac481</t>
         </is>
       </c>
       <c r="F131" s="3" t="inlineStr">
         <is>
-          <t>Prove Q21 REJECTS an answer that breaks its rule. The QRE's rule is: the answer must be at least 5 characters; the answer must be at most 500 characters</t>
+          <t>Prove Q21 refuses to let the respondent past when it is left blank. The questionnaire marks it compulsory, and it is a text question</t>
         </is>
       </c>
       <c r="G131" s="3" t="inlineStr">
@@ -9713,17 +9713,18 @@
       </c>
       <c r="H131" s="3" t="inlineStr">
         <is>
-          <t>At Q21, type “O'Brien said "yes" &lt;50% &amp; more”, then submit.</t>
+          <t>At Q21, type 3 spaces and nothing else, then submit.</t>
         </is>
       </c>
       <c r="I131" s="3" t="inlineStr">
         <is>
-          <t>1. the survey ACCEPTS the answer and moves to the next page</t>
+          <t>1. the survey REFUSES to move on; the same page reappears
+2. an error message is shown against Q21</t>
         </is>
       </c>
       <c r="J131" s="2" t="inlineStr">
         <is>
-          <t>Answer rule accepts or rejects</t>
+          <t>Blank answer is blocked</t>
         </is>
       </c>
       <c r="K131" s="2" t="inlineStr">
@@ -9738,12 +9739,12 @@
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>Q21</t>
+          <t>DT3</t>
         </is>
       </c>
       <c r="C132" s="3" t="inlineStr">
         <is>
-          <t>Q21 | What most influenced your choice? | text | — | Validate: {"min_length": 5, "max_length": 500}</t>
+          <t>DT3 | You're almost done! Thank you for your answers. Just a few last questions about you to finish up. | text display | — | Always show</t>
         </is>
       </c>
       <c r="D132" s="2" t="inlineStr">
@@ -9753,92 +9754,15 @@
       </c>
       <c r="E132" s="2" t="inlineStr">
         <is>
-          <t>TC-2b316ac481</t>
+          <t>TC-60f46acb6d</t>
         </is>
       </c>
       <c r="F132" s="3" t="inlineStr">
         <is>
-          <t>Prove Q21 refuses to let the respondent past when it is left blank. The questionnaire marks it compulsory, and it is a text question</t>
+          <t>Prove the survey flows correctly at DT3: answer it normally and the respondent should move on to whatever the questionnaire says comes next, not stop or jump elsewhere</t>
         </is>
       </c>
       <c r="G132" s="3" t="inlineStr">
-        <is>
-          <t>1. S1 = Yes
-2. S2 = Personally manage an ongoing chronic health condition
-3. S3 = No
-4. S4 = No
-5. Q1 = Care Network A
-6. Q2 = Care Network A
-7. Q3 = Care Network A
-8. Q4 = Recently diagnosed
-9. Q5 = Primary-care physician
-10. Q6 = Primary-care physician
-11. Q7 = Very poor
-12. Q8 = 0
-13. Q9 = Q9-R1=Very poor; Q9-R2=Very poor; Q9-R3=Very poor...
-14. Q10 = Yes
-15. Q11 = Phone
-16. Q12 = Fully
-17. Q13 = Very low
-18. Q15 = Yes
-19. Q16 = Price
-20. Q18 = Price=20; Quality=20; Convenience=20...
-21. Q19 = Concept A
-22. Q20 = Very poor</t>
-        </is>
-      </c>
-      <c r="H132" s="3" t="inlineStr">
-        <is>
-          <t>At Q21, type 3 spaces and nothing else, then submit.</t>
-        </is>
-      </c>
-      <c r="I132" s="3" t="inlineStr">
-        <is>
-          <t>1. the survey REFUSES to move on; the same page reappears
-2. an error message is shown against Q21</t>
-        </is>
-      </c>
-      <c r="J132" s="2" t="inlineStr">
-        <is>
-          <t>Blank answer is blocked</t>
-        </is>
-      </c>
-      <c r="K132" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" s="2" t="n">
-        <v>132</v>
-      </c>
-      <c r="B133" s="2" t="inlineStr">
-        <is>
-          <t>DT3</t>
-        </is>
-      </c>
-      <c r="C133" s="3" t="inlineStr">
-        <is>
-          <t>DT3 | You're almost done! Thank you for your answers. Just a few last questions about you to finish up. | text display | — | Always show</t>
-        </is>
-      </c>
-      <c r="D133" s="2" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="E133" s="2" t="inlineStr">
-        <is>
-          <t>TC-60f46acb6d</t>
-        </is>
-      </c>
-      <c r="F133" s="3" t="inlineStr">
-        <is>
-          <t>Prove the survey flows correctly at DT3: answer it normally and the respondent should move on to whatever the questionnaire says comes next, not stop or jump elsewhere</t>
-        </is>
-      </c>
-      <c r="G133" s="3" t="inlineStr">
         <is>
           <t>1. S1 = Yes
 2. S2 = Personally manage an ongoing chronic health condition
@@ -9870,57 +9794,57 @@
 28. Q22 = Yes</t>
         </is>
       </c>
-      <c r="H133" s="3" t="inlineStr">
+      <c r="H132" s="3" t="inlineStr">
         <is>
           <t>Answer through the whole survey as listed, then observe where it ends.</t>
         </is>
       </c>
-      <c r="I133" s="3" t="inlineStr">
+      <c r="I132" s="3" t="inlineStr">
         <is>
           <t>1. the next question shown is D1</t>
         </is>
       </c>
-      <c r="J133" s="2" t="inlineStr">
+      <c r="J132" s="2" t="inlineStr">
         <is>
           <t>Shows / hides correctly</t>
         </is>
       </c>
-      <c r="K133" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" s="2" t="n">
-        <v>133</v>
-      </c>
-      <c r="B134" s="2" t="inlineStr">
+      <c r="K132" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="n">
+        <v>132</v>
+      </c>
+      <c r="B133" s="2" t="inlineStr">
         <is>
           <t>D1</t>
         </is>
       </c>
-      <c r="C134" s="3" t="inlineStr">
+      <c r="C133" s="3" t="inlineStr">
         <is>
           <t>D1 | Which region do you live in? | single | North; South; East; West; Central | Always show</t>
         </is>
       </c>
-      <c r="D134" s="2" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="E134" s="2" t="inlineStr">
+      <c r="D133" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E133" s="2" t="inlineStr">
         <is>
           <t>TC-9d345eef73</t>
         </is>
       </c>
-      <c r="F134" s="3" t="inlineStr">
+      <c r="F133" s="3" t="inlineStr">
         <is>
           <t>Prove the survey flows correctly at D1: answer it normally and the respondent should move on to whatever the questionnaire says comes next, not stop or jump elsewhere</t>
         </is>
       </c>
-      <c r="G134" s="3" t="inlineStr">
+      <c r="G133" s="3" t="inlineStr">
         <is>
           <t>1. S1 = Yes
 2. S2 = Personally manage an ongoing chronic health condition
@@ -9952,58 +9876,58 @@
 28. Q22 = Yes</t>
         </is>
       </c>
-      <c r="H134" s="3" t="inlineStr">
+      <c r="H133" s="3" t="inlineStr">
         <is>
           <t>Answer through the whole survey as listed, then observe where it ends.</t>
         </is>
       </c>
-      <c r="I134" s="3" t="inlineStr">
+      <c r="I133" s="3" t="inlineStr">
         <is>
           <t>1. D1 IS shown on the page
 2. the next question shown is D2</t>
         </is>
       </c>
-      <c r="J134" s="2" t="inlineStr">
+      <c r="J133" s="2" t="inlineStr">
         <is>
           <t>Shows / hides correctly</t>
         </is>
       </c>
-      <c r="K134" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" s="2" t="n">
-        <v>134</v>
-      </c>
-      <c r="B135" s="2" t="inlineStr">
+      <c r="K133" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="n">
+        <v>133</v>
+      </c>
+      <c r="B134" s="2" t="inlineStr">
         <is>
           <t>D1</t>
         </is>
       </c>
-      <c r="C135" s="3" t="inlineStr">
+      <c r="C134" s="3" t="inlineStr">
         <is>
           <t>D1 | Which region do you live in? | single | North; South; East; West; Central | Always show</t>
         </is>
       </c>
-      <c r="D135" s="2" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="E135" s="2" t="inlineStr">
+      <c r="D134" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E134" s="2" t="inlineStr">
         <is>
           <t>TC-eba66f169b</t>
         </is>
       </c>
-      <c r="F135" s="3" t="inlineStr">
+      <c r="F134" s="3" t="inlineStr">
         <is>
           <t>Prove D1 refuses to let the respondent past when it is left blank. The questionnaire marks it compulsory, and it is a single question</t>
         </is>
       </c>
-      <c r="G135" s="3" t="inlineStr">
+      <c r="G134" s="3" t="inlineStr">
         <is>
           <t>1. S1 = Yes
 2. S2 = Personally manage an ongoing chronic health condition
@@ -10030,58 +9954,58 @@
 23. Q21 = xxxxx</t>
         </is>
       </c>
-      <c r="H135" s="3" t="inlineStr">
+      <c r="H134" s="3" t="inlineStr">
         <is>
           <t>At D1, select nothing at all, then submit.</t>
         </is>
       </c>
-      <c r="I135" s="3" t="inlineStr">
+      <c r="I134" s="3" t="inlineStr">
         <is>
           <t>1. the survey REFUSES to move on; the same page reappears
 2. an error message is shown against D1</t>
         </is>
       </c>
-      <c r="J135" s="2" t="inlineStr">
+      <c r="J134" s="2" t="inlineStr">
         <is>
           <t>Blank answer is blocked</t>
         </is>
       </c>
-      <c r="K135" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" s="2" t="n">
-        <v>135</v>
-      </c>
-      <c r="B136" s="2" t="inlineStr">
+      <c r="K134" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="n">
+        <v>134</v>
+      </c>
+      <c r="B135" s="2" t="inlineStr">
         <is>
           <t>D1</t>
         </is>
       </c>
-      <c r="C136" s="3" t="inlineStr">
+      <c r="C135" s="3" t="inlineStr">
         <is>
           <t>D1 | Which region do you live in? | single | North; South; East; West; Central | Always show</t>
         </is>
       </c>
-      <c r="D136" s="2" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="E136" s="2" t="inlineStr">
+      <c r="D135" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E135" s="2" t="inlineStr">
         <is>
           <t>TC-640f339984</t>
         </is>
       </c>
-      <c r="F136" s="3" t="inlineStr">
+      <c r="F135" s="3" t="inlineStr">
         <is>
           <t>Prove quota QUOTA_REGION lets a 'North' respondent through while that group is still below its target</t>
         </is>
       </c>
-      <c r="G136" s="3" t="inlineStr">
+      <c r="G135" s="3" t="inlineStr">
         <is>
           <t>1. S1 = Yes
 2. S2 = Personally manage an ongoing chronic health condition
@@ -10108,57 +10032,57 @@
 23. Q21 = xxxxx</t>
         </is>
       </c>
-      <c r="H136" s="3" t="inlineStr">
+      <c r="H135" s="3" t="inlineStr">
         <is>
           <t>At D1, choose “North”, then submit.</t>
         </is>
       </c>
-      <c r="I136" s="3" t="inlineStr">
+      <c r="I135" s="3" t="inlineStr">
         <is>
           <t>1. the respondent is allowed to continue, not sent to the quota-full ending</t>
         </is>
       </c>
-      <c r="J136" s="2" t="inlineStr">
+      <c r="J135" s="2" t="inlineStr">
         <is>
           <t>Quota accepts or turns away</t>
         </is>
       </c>
-      <c r="K136" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" s="2" t="n">
-        <v>136</v>
-      </c>
-      <c r="B137" s="2" t="inlineStr">
+      <c r="K135" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="n">
+        <v>135</v>
+      </c>
+      <c r="B136" s="2" t="inlineStr">
         <is>
           <t>D1</t>
         </is>
       </c>
-      <c r="C137" s="3" t="inlineStr">
+      <c r="C136" s="3" t="inlineStr">
         <is>
           <t>D1 | Which region do you live in? | single | North; South; East; West; Central | Always show</t>
         </is>
       </c>
-      <c r="D137" s="2" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="E137" s="2" t="inlineStr">
+      <c r="D136" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E136" s="2" t="inlineStr">
         <is>
           <t>TC-6a4f70dee1</t>
         </is>
       </c>
-      <c r="F137" s="3" t="inlineStr">
+      <c r="F136" s="3" t="inlineStr">
         <is>
           <t>Prove quota QUOTA_REGION lets a 'South' respondent through while that group is still below its target</t>
         </is>
       </c>
-      <c r="G137" s="3" t="inlineStr">
+      <c r="G136" s="3" t="inlineStr">
         <is>
           <t>1. S1 = Yes
 2. S2 = Personally manage an ongoing chronic health condition
@@ -10185,57 +10109,57 @@
 23. Q21 = xxxxx</t>
         </is>
       </c>
-      <c r="H137" s="3" t="inlineStr">
+      <c r="H136" s="3" t="inlineStr">
         <is>
           <t>At D1, choose “South”, then submit.</t>
         </is>
       </c>
-      <c r="I137" s="3" t="inlineStr">
+      <c r="I136" s="3" t="inlineStr">
         <is>
           <t>1. the respondent is allowed to continue, not sent to the quota-full ending</t>
         </is>
       </c>
-      <c r="J137" s="2" t="inlineStr">
+      <c r="J136" s="2" t="inlineStr">
         <is>
           <t>Quota accepts or turns away</t>
         </is>
       </c>
-      <c r="K137" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" s="2" t="n">
-        <v>137</v>
-      </c>
-      <c r="B138" s="2" t="inlineStr">
+      <c r="K136" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="n">
+        <v>136</v>
+      </c>
+      <c r="B137" s="2" t="inlineStr">
         <is>
           <t>D1</t>
         </is>
       </c>
-      <c r="C138" s="3" t="inlineStr">
+      <c r="C137" s="3" t="inlineStr">
         <is>
           <t>D1 | Which region do you live in? | single | North; South; East; West; Central | Always show</t>
         </is>
       </c>
-      <c r="D138" s="2" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="E138" s="2" t="inlineStr">
+      <c r="D137" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E137" s="2" t="inlineStr">
         <is>
           <t>TC-add22f59a7</t>
         </is>
       </c>
-      <c r="F138" s="3" t="inlineStr">
+      <c r="F137" s="3" t="inlineStr">
         <is>
           <t>Prove quota QUOTA_REGION lets a 'East' respondent through while that group is still below its target</t>
         </is>
       </c>
-      <c r="G138" s="3" t="inlineStr">
+      <c r="G137" s="3" t="inlineStr">
         <is>
           <t>1. S1 = Yes
 2. S2 = Personally manage an ongoing chronic health condition
@@ -10262,57 +10186,57 @@
 23. Q21 = xxxxx</t>
         </is>
       </c>
-      <c r="H138" s="3" t="inlineStr">
+      <c r="H137" s="3" t="inlineStr">
         <is>
           <t>At D1, choose “East”, then submit.</t>
         </is>
       </c>
-      <c r="I138" s="3" t="inlineStr">
+      <c r="I137" s="3" t="inlineStr">
         <is>
           <t>1. the respondent is allowed to continue, not sent to the quota-full ending</t>
         </is>
       </c>
-      <c r="J138" s="2" t="inlineStr">
+      <c r="J137" s="2" t="inlineStr">
         <is>
           <t>Quota accepts or turns away</t>
         </is>
       </c>
-      <c r="K138" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" s="2" t="n">
-        <v>138</v>
-      </c>
-      <c r="B139" s="2" t="inlineStr">
+      <c r="K137" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="n">
+        <v>137</v>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
         <is>
           <t>D1</t>
         </is>
       </c>
-      <c r="C139" s="3" t="inlineStr">
+      <c r="C138" s="3" t="inlineStr">
         <is>
           <t>D1 | Which region do you live in? | single | North; South; East; West; Central | Always show</t>
         </is>
       </c>
-      <c r="D139" s="2" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="E139" s="2" t="inlineStr">
+      <c r="D138" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E138" s="2" t="inlineStr">
         <is>
           <t>TC-e3f1efd2fe</t>
         </is>
       </c>
-      <c r="F139" s="3" t="inlineStr">
+      <c r="F138" s="3" t="inlineStr">
         <is>
           <t>Prove quota QUOTA_REGION lets a 'West' respondent through while that group is still below its target</t>
         </is>
       </c>
-      <c r="G139" s="3" t="inlineStr">
+      <c r="G138" s="3" t="inlineStr">
         <is>
           <t>1. S1 = Yes
 2. S2 = Personally manage an ongoing chronic health condition
@@ -10339,57 +10263,57 @@
 23. Q21 = xxxxx</t>
         </is>
       </c>
-      <c r="H139" s="3" t="inlineStr">
+      <c r="H138" s="3" t="inlineStr">
         <is>
           <t>At D1, choose “West”, then submit.</t>
         </is>
       </c>
-      <c r="I139" s="3" t="inlineStr">
+      <c r="I138" s="3" t="inlineStr">
         <is>
           <t>1. the respondent is allowed to continue, not sent to the quota-full ending</t>
         </is>
       </c>
-      <c r="J139" s="2" t="inlineStr">
+      <c r="J138" s="2" t="inlineStr">
         <is>
           <t>Quota accepts or turns away</t>
         </is>
       </c>
-      <c r="K139" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" s="2" t="n">
-        <v>139</v>
-      </c>
-      <c r="B140" s="2" t="inlineStr">
+      <c r="K138" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="n">
+        <v>138</v>
+      </c>
+      <c r="B139" s="2" t="inlineStr">
         <is>
           <t>D1</t>
         </is>
       </c>
-      <c r="C140" s="3" t="inlineStr">
+      <c r="C139" s="3" t="inlineStr">
         <is>
           <t>D1 | Which region do you live in? | single | North; South; East; West; Central | Always show</t>
         </is>
       </c>
-      <c r="D140" s="2" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="E140" s="2" t="inlineStr">
+      <c r="D139" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E139" s="2" t="inlineStr">
         <is>
           <t>TC-faf234994c</t>
         </is>
       </c>
-      <c r="F140" s="3" t="inlineStr">
+      <c r="F139" s="3" t="inlineStr">
         <is>
           <t>Prove quota QUOTA_REGION lets a 'Central' respondent through while that group is still below its target</t>
         </is>
       </c>
-      <c r="G140" s="3" t="inlineStr">
+      <c r="G139" s="3" t="inlineStr">
         <is>
           <t>1. S1 = Yes
 2. S2 = Personally manage an ongoing chronic health condition
@@ -10416,57 +10340,57 @@
 23. Q21 = xxxxx</t>
         </is>
       </c>
-      <c r="H140" s="3" t="inlineStr">
+      <c r="H139" s="3" t="inlineStr">
         <is>
           <t>At D1, choose “Central”, then submit.</t>
         </is>
       </c>
-      <c r="I140" s="3" t="inlineStr">
+      <c r="I139" s="3" t="inlineStr">
         <is>
           <t>1. the respondent is allowed to continue, not sent to the quota-full ending</t>
         </is>
       </c>
-      <c r="J140" s="2" t="inlineStr">
+      <c r="J139" s="2" t="inlineStr">
         <is>
           <t>Quota accepts or turns away</t>
         </is>
       </c>
-      <c r="K140" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" s="2" t="n">
-        <v>140</v>
-      </c>
-      <c r="B141" s="2" t="inlineStr">
+      <c r="K139" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="n">
+        <v>139</v>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
         <is>
           <t>D2</t>
         </is>
       </c>
-      <c r="C141" s="3" t="inlineStr">
+      <c r="C140" s="3" t="inlineStr">
         <is>
           <t>D2 | Which age group describes you? | single | 21-29; 30-39; 40-49; 50-59; 60+ | Always show</t>
         </is>
       </c>
-      <c r="D141" s="2" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="E141" s="2" t="inlineStr">
+      <c r="D140" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E140" s="2" t="inlineStr">
         <is>
           <t>TC-a1ac064e4d</t>
         </is>
       </c>
-      <c r="F141" s="3" t="inlineStr">
+      <c r="F140" s="3" t="inlineStr">
         <is>
           <t>Prove the survey flows correctly at D2: answer it normally and the respondent should move on to whatever the questionnaire says comes next, not stop or jump elsewhere</t>
         </is>
       </c>
-      <c r="G141" s="3" t="inlineStr">
+      <c r="G140" s="3" t="inlineStr">
         <is>
           <t>1. S1 = Yes
 2. S2 = Personally manage an ongoing chronic health condition
@@ -10498,58 +10422,58 @@
 28. Q22 = Yes</t>
         </is>
       </c>
-      <c r="H141" s="3" t="inlineStr">
+      <c r="H140" s="3" t="inlineStr">
         <is>
           <t>Answer through the whole survey as listed, then observe where it ends.</t>
         </is>
       </c>
-      <c r="I141" s="3" t="inlineStr">
+      <c r="I140" s="3" t="inlineStr">
         <is>
           <t>1. D2 IS shown on the page
 2. the next question shown is D3</t>
         </is>
       </c>
-      <c r="J141" s="2" t="inlineStr">
+      <c r="J140" s="2" t="inlineStr">
         <is>
           <t>Shows / hides correctly</t>
         </is>
       </c>
-      <c r="K141" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" s="2" t="n">
-        <v>141</v>
-      </c>
-      <c r="B142" s="2" t="inlineStr">
+      <c r="K140" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="n">
+        <v>140</v>
+      </c>
+      <c r="B141" s="2" t="inlineStr">
         <is>
           <t>D2</t>
         </is>
       </c>
-      <c r="C142" s="3" t="inlineStr">
+      <c r="C141" s="3" t="inlineStr">
         <is>
           <t>D2 | Which age group describes you? | single | 21-29; 30-39; 40-49; 50-59; 60+ | Always show</t>
         </is>
       </c>
-      <c r="D142" s="2" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="E142" s="2" t="inlineStr">
+      <c r="D141" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E141" s="2" t="inlineStr">
         <is>
           <t>TC-e3d95ddd0a</t>
         </is>
       </c>
-      <c r="F142" s="3" t="inlineStr">
+      <c r="F141" s="3" t="inlineStr">
         <is>
           <t>Prove D2 refuses to let the respondent past when it is left blank. The questionnaire marks it compulsory, and it is a single question</t>
         </is>
       </c>
-      <c r="G142" s="3" t="inlineStr">
+      <c r="G141" s="3" t="inlineStr">
         <is>
           <t>1. S1 = Yes
 2. S2 = Personally manage an ongoing chronic health condition
@@ -10577,58 +10501,58 @@
 24. D1 = North</t>
         </is>
       </c>
-      <c r="H142" s="3" t="inlineStr">
+      <c r="H141" s="3" t="inlineStr">
         <is>
           <t>At D2, select nothing at all, then submit.</t>
         </is>
       </c>
-      <c r="I142" s="3" t="inlineStr">
+      <c r="I141" s="3" t="inlineStr">
         <is>
           <t>1. the survey REFUSES to move on; the same page reappears
 2. an error message is shown against D2</t>
         </is>
       </c>
-      <c r="J142" s="2" t="inlineStr">
+      <c r="J141" s="2" t="inlineStr">
         <is>
           <t>Blank answer is blocked</t>
         </is>
       </c>
-      <c r="K142" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" s="2" t="n">
-        <v>142</v>
-      </c>
-      <c r="B143" s="2" t="inlineStr">
+      <c r="K141" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="n">
+        <v>141</v>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
         <is>
           <t>D2</t>
         </is>
       </c>
-      <c r="C143" s="3" t="inlineStr">
+      <c r="C142" s="3" t="inlineStr">
         <is>
           <t>D2 | Which age group describes you? | single | 21-29; 30-39; 40-49; 50-59; 60+ | Always show</t>
         </is>
       </c>
-      <c r="D143" s="2" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="E143" s="2" t="inlineStr">
+      <c r="D142" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E142" s="2" t="inlineStr">
         <is>
           <t>TC-9e12b71968</t>
         </is>
       </c>
-      <c r="F143" s="3" t="inlineStr">
+      <c r="F142" s="3" t="inlineStr">
         <is>
           <t>Prove quota QUOTA_AGE lets a '21-29' respondent through while that group is still below its target</t>
         </is>
       </c>
-      <c r="G143" s="3" t="inlineStr">
+      <c r="G142" s="3" t="inlineStr">
         <is>
           <t>1. S1 = Yes
 2. S2 = Personally manage an ongoing chronic health condition
@@ -10656,57 +10580,57 @@
 24. D1 = North</t>
         </is>
       </c>
-      <c r="H143" s="3" t="inlineStr">
+      <c r="H142" s="3" t="inlineStr">
         <is>
           <t>At D2, choose “21-29”, then submit.</t>
         </is>
       </c>
-      <c r="I143" s="3" t="inlineStr">
+      <c r="I142" s="3" t="inlineStr">
         <is>
           <t>1. the respondent is allowed to continue, not sent to the quota-full ending</t>
         </is>
       </c>
-      <c r="J143" s="2" t="inlineStr">
+      <c r="J142" s="2" t="inlineStr">
         <is>
           <t>Quota accepts or turns away</t>
         </is>
       </c>
-      <c r="K143" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" s="2" t="n">
-        <v>143</v>
-      </c>
-      <c r="B144" s="2" t="inlineStr">
+      <c r="K142" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="n">
+        <v>142</v>
+      </c>
+      <c r="B143" s="2" t="inlineStr">
         <is>
           <t>D2</t>
         </is>
       </c>
-      <c r="C144" s="3" t="inlineStr">
+      <c r="C143" s="3" t="inlineStr">
         <is>
           <t>D2 | Which age group describes you? | single | 21-29; 30-39; 40-49; 50-59; 60+ | Always show</t>
         </is>
       </c>
-      <c r="D144" s="2" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="E144" s="2" t="inlineStr">
+      <c r="D143" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E143" s="2" t="inlineStr">
         <is>
           <t>TC-6c5662fab4</t>
         </is>
       </c>
-      <c r="F144" s="3" t="inlineStr">
+      <c r="F143" s="3" t="inlineStr">
         <is>
           <t>Prove quota QUOTA_AGE lets a '30-39' respondent through while that group is still below its target</t>
         </is>
       </c>
-      <c r="G144" s="3" t="inlineStr">
+      <c r="G143" s="3" t="inlineStr">
         <is>
           <t>1. S1 = Yes
 2. S2 = Personally manage an ongoing chronic health condition
@@ -10734,57 +10658,57 @@
 24. D1 = North</t>
         </is>
       </c>
-      <c r="H144" s="3" t="inlineStr">
+      <c r="H143" s="3" t="inlineStr">
         <is>
           <t>At D2, choose “30-39”, then submit.</t>
         </is>
       </c>
-      <c r="I144" s="3" t="inlineStr">
+      <c r="I143" s="3" t="inlineStr">
         <is>
           <t>1. the respondent is allowed to continue, not sent to the quota-full ending</t>
         </is>
       </c>
-      <c r="J144" s="2" t="inlineStr">
+      <c r="J143" s="2" t="inlineStr">
         <is>
           <t>Quota accepts or turns away</t>
         </is>
       </c>
-      <c r="K144" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" s="2" t="n">
-        <v>144</v>
-      </c>
-      <c r="B145" s="2" t="inlineStr">
+      <c r="K143" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="n">
+        <v>143</v>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
         <is>
           <t>D2</t>
         </is>
       </c>
-      <c r="C145" s="3" t="inlineStr">
+      <c r="C144" s="3" t="inlineStr">
         <is>
           <t>D2 | Which age group describes you? | single | 21-29; 30-39; 40-49; 50-59; 60+ | Always show</t>
         </is>
       </c>
-      <c r="D145" s="2" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="E145" s="2" t="inlineStr">
+      <c r="D144" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E144" s="2" t="inlineStr">
         <is>
           <t>TC-dd41da385a</t>
         </is>
       </c>
-      <c r="F145" s="3" t="inlineStr">
+      <c r="F144" s="3" t="inlineStr">
         <is>
           <t>Prove quota QUOTA_AGE lets a '40-49' respondent through while that group is still below its target</t>
         </is>
       </c>
-      <c r="G145" s="3" t="inlineStr">
+      <c r="G144" s="3" t="inlineStr">
         <is>
           <t>1. S1 = Yes
 2. S2 = Personally manage an ongoing chronic health condition
@@ -10812,57 +10736,57 @@
 24. D1 = North</t>
         </is>
       </c>
-      <c r="H145" s="3" t="inlineStr">
+      <c r="H144" s="3" t="inlineStr">
         <is>
           <t>At D2, choose “40-49”, then submit.</t>
         </is>
       </c>
-      <c r="I145" s="3" t="inlineStr">
+      <c r="I144" s="3" t="inlineStr">
         <is>
           <t>1. the respondent is allowed to continue, not sent to the quota-full ending</t>
         </is>
       </c>
-      <c r="J145" s="2" t="inlineStr">
+      <c r="J144" s="2" t="inlineStr">
         <is>
           <t>Quota accepts or turns away</t>
         </is>
       </c>
-      <c r="K145" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" s="2" t="n">
-        <v>145</v>
-      </c>
-      <c r="B146" s="2" t="inlineStr">
+      <c r="K144" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="n">
+        <v>144</v>
+      </c>
+      <c r="B145" s="2" t="inlineStr">
         <is>
           <t>D2</t>
         </is>
       </c>
-      <c r="C146" s="3" t="inlineStr">
+      <c r="C145" s="3" t="inlineStr">
         <is>
           <t>D2 | Which age group describes you? | single | 21-29; 30-39; 40-49; 50-59; 60+ | Always show</t>
         </is>
       </c>
-      <c r="D146" s="2" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="E146" s="2" t="inlineStr">
+      <c r="D145" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E145" s="2" t="inlineStr">
         <is>
           <t>TC-d79d3aefa5</t>
         </is>
       </c>
-      <c r="F146" s="3" t="inlineStr">
+      <c r="F145" s="3" t="inlineStr">
         <is>
           <t>Prove quota QUOTA_AGE lets a '50-59' respondent through while that group is still below its target</t>
         </is>
       </c>
-      <c r="G146" s="3" t="inlineStr">
+      <c r="G145" s="3" t="inlineStr">
         <is>
           <t>1. S1 = Yes
 2. S2 = Personally manage an ongoing chronic health condition
@@ -10890,57 +10814,57 @@
 24. D1 = North</t>
         </is>
       </c>
-      <c r="H146" s="3" t="inlineStr">
+      <c r="H145" s="3" t="inlineStr">
         <is>
           <t>At D2, choose “50-59”, then submit.</t>
         </is>
       </c>
-      <c r="I146" s="3" t="inlineStr">
+      <c r="I145" s="3" t="inlineStr">
         <is>
           <t>1. the respondent is allowed to continue, not sent to the quota-full ending</t>
         </is>
       </c>
-      <c r="J146" s="2" t="inlineStr">
+      <c r="J145" s="2" t="inlineStr">
         <is>
           <t>Quota accepts or turns away</t>
         </is>
       </c>
-      <c r="K146" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" s="2" t="n">
-        <v>146</v>
-      </c>
-      <c r="B147" s="2" t="inlineStr">
+      <c r="K145" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="n">
+        <v>145</v>
+      </c>
+      <c r="B146" s="2" t="inlineStr">
         <is>
           <t>D2</t>
         </is>
       </c>
-      <c r="C147" s="3" t="inlineStr">
+      <c r="C146" s="3" t="inlineStr">
         <is>
           <t>D2 | Which age group describes you? | single | 21-29; 30-39; 40-49; 50-59; 60+ | Always show</t>
         </is>
       </c>
-      <c r="D147" s="2" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="E147" s="2" t="inlineStr">
+      <c r="D146" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E146" s="2" t="inlineStr">
         <is>
           <t>TC-718cbe9fd7</t>
         </is>
       </c>
-      <c r="F147" s="3" t="inlineStr">
+      <c r="F146" s="3" t="inlineStr">
         <is>
           <t>Prove quota QUOTA_AGE lets a '60+' respondent through while that group is still below its target</t>
         </is>
       </c>
-      <c r="G147" s="3" t="inlineStr">
+      <c r="G146" s="3" t="inlineStr">
         <is>
           <t>1. S1 = Yes
 2. S2 = Personally manage an ongoing chronic health condition
@@ -10968,57 +10892,57 @@
 24. D1 = North</t>
         </is>
       </c>
-      <c r="H147" s="3" t="inlineStr">
+      <c r="H146" s="3" t="inlineStr">
         <is>
           <t>At D2, choose “60+”, then submit.</t>
         </is>
       </c>
-      <c r="I147" s="3" t="inlineStr">
+      <c r="I146" s="3" t="inlineStr">
         <is>
           <t>1. the respondent is allowed to continue, not sent to the quota-full ending</t>
         </is>
       </c>
-      <c r="J147" s="2" t="inlineStr">
+      <c r="J146" s="2" t="inlineStr">
         <is>
           <t>Quota accepts or turns away</t>
         </is>
       </c>
-      <c r="K147" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" s="2" t="n">
-        <v>147</v>
-      </c>
-      <c r="B148" s="2" t="inlineStr">
+      <c r="K146" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="n">
+        <v>146</v>
+      </c>
+      <c r="B147" s="2" t="inlineStr">
         <is>
           <t>D3</t>
         </is>
       </c>
-      <c r="C148" s="3" t="inlineStr">
+      <c r="C147" s="3" t="inlineStr">
         <is>
           <t>D3 | How do you describe your gender? | single | Woman; Man; Non-binary; Prefer to self-describe; Prefer not to say | Always show</t>
         </is>
       </c>
-      <c r="D148" s="2" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="E148" s="2" t="inlineStr">
+      <c r="D147" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E147" s="2" t="inlineStr">
         <is>
           <t>TC-531a6544ed</t>
         </is>
       </c>
-      <c r="F148" s="3" t="inlineStr">
+      <c r="F147" s="3" t="inlineStr">
         <is>
           <t>Prove the survey flows correctly at D3: answer it normally and the respondent should move on to whatever the questionnaire says comes next, not stop or jump elsewhere</t>
         </is>
       </c>
-      <c r="G148" s="3" t="inlineStr">
+      <c r="G147" s="3" t="inlineStr">
         <is>
           <t>1. S1 = Yes
 2. S2 = Personally manage an ongoing chronic health condition
@@ -11050,58 +10974,58 @@
 28. Q22 = Yes</t>
         </is>
       </c>
-      <c r="H148" s="3" t="inlineStr">
+      <c r="H147" s="3" t="inlineStr">
         <is>
           <t>Answer through the whole survey as listed, then observe where it ends.</t>
         </is>
       </c>
-      <c r="I148" s="3" t="inlineStr">
+      <c r="I147" s="3" t="inlineStr">
         <is>
           <t>1. D3 IS shown on the page
 2. the next question shown is D4</t>
         </is>
       </c>
-      <c r="J148" s="2" t="inlineStr">
+      <c r="J147" s="2" t="inlineStr">
         <is>
           <t>Shows / hides correctly</t>
         </is>
       </c>
-      <c r="K148" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" s="2" t="n">
-        <v>148</v>
-      </c>
-      <c r="B149" s="2" t="inlineStr">
+      <c r="K147" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="n">
+        <v>147</v>
+      </c>
+      <c r="B148" s="2" t="inlineStr">
         <is>
           <t>D3</t>
         </is>
       </c>
-      <c r="C149" s="3" t="inlineStr">
+      <c r="C148" s="3" t="inlineStr">
         <is>
           <t>D3 | How do you describe your gender? | single | Woman; Man; Non-binary; Prefer to self-describe; Prefer not to say | Always show</t>
         </is>
       </c>
-      <c r="D149" s="2" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="E149" s="2" t="inlineStr">
+      <c r="D148" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E148" s="2" t="inlineStr">
         <is>
           <t>TC-799f9fd202</t>
         </is>
       </c>
-      <c r="F149" s="3" t="inlineStr">
+      <c r="F148" s="3" t="inlineStr">
         <is>
           <t>Prove D3 refuses to let the respondent past when it is left blank. The questionnaire marks it compulsory, and it is a single question</t>
         </is>
       </c>
-      <c r="G149" s="3" t="inlineStr">
+      <c r="G148" s="3" t="inlineStr">
         <is>
           <t>1. S1 = Yes
 2. S2 = Personally manage an ongoing chronic health condition
@@ -11130,58 +11054,58 @@
 25. D2 = 21-29</t>
         </is>
       </c>
-      <c r="H149" s="3" t="inlineStr">
+      <c r="H148" s="3" t="inlineStr">
         <is>
           <t>At D3, select nothing at all, then submit.</t>
         </is>
       </c>
-      <c r="I149" s="3" t="inlineStr">
+      <c r="I148" s="3" t="inlineStr">
         <is>
           <t>1. the survey REFUSES to move on; the same page reappears
 2. an error message is shown against D3</t>
         </is>
       </c>
-      <c r="J149" s="2" t="inlineStr">
+      <c r="J148" s="2" t="inlineStr">
         <is>
           <t>Blank answer is blocked</t>
         </is>
       </c>
-      <c r="K149" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" s="2" t="n">
-        <v>149</v>
-      </c>
-      <c r="B150" s="2" t="inlineStr">
+      <c r="K148" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="n">
+        <v>148</v>
+      </c>
+      <c r="B149" s="2" t="inlineStr">
         <is>
           <t>D4</t>
         </is>
       </c>
-      <c r="C150" s="3" t="inlineStr">
+      <c r="C149" s="3" t="inlineStr">
         <is>
           <t>D4 | What is your household or organizational decision band? | single | Band 1; Band 2; Band 3; Band 4; Prefer not to say | Always show</t>
         </is>
       </c>
-      <c r="D150" s="2" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="E150" s="2" t="inlineStr">
+      <c r="D149" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E149" s="2" t="inlineStr">
         <is>
           <t>TC-0c2ebe3557</t>
         </is>
       </c>
-      <c r="F150" s="3" t="inlineStr">
+      <c r="F149" s="3" t="inlineStr">
         <is>
           <t>Prove the survey flows correctly at D4: answer it normally and the respondent should move on to whatever the questionnaire says comes next, not stop or jump elsewhere</t>
         </is>
       </c>
-      <c r="G150" s="3" t="inlineStr">
+      <c r="G149" s="3" t="inlineStr">
         <is>
           <t>1. S1 = Yes
 2. S2 = Personally manage an ongoing chronic health condition
@@ -11213,58 +11137,58 @@
 28. Q22 = Yes</t>
         </is>
       </c>
-      <c r="H150" s="3" t="inlineStr">
+      <c r="H149" s="3" t="inlineStr">
         <is>
           <t>Answer through the whole survey as listed, then observe where it ends.</t>
         </is>
       </c>
-      <c r="I150" s="3" t="inlineStr">
+      <c r="I149" s="3" t="inlineStr">
         <is>
           <t>1. D4 IS shown on the page
 2. the next question shown is Q22</t>
         </is>
       </c>
-      <c r="J150" s="2" t="inlineStr">
+      <c r="J149" s="2" t="inlineStr">
         <is>
           <t>Shows / hides correctly</t>
         </is>
       </c>
-      <c r="K150" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" s="2" t="n">
-        <v>150</v>
-      </c>
-      <c r="B151" s="2" t="inlineStr">
+      <c r="K149" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="n">
+        <v>149</v>
+      </c>
+      <c r="B150" s="2" t="inlineStr">
         <is>
           <t>D4</t>
         </is>
       </c>
-      <c r="C151" s="3" t="inlineStr">
+      <c r="C150" s="3" t="inlineStr">
         <is>
           <t>D4 | What is your household or organizational decision band? | single | Band 1; Band 2; Band 3; Band 4; Prefer not to say | Always show</t>
         </is>
       </c>
-      <c r="D151" s="2" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="E151" s="2" t="inlineStr">
+      <c r="D150" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E150" s="2" t="inlineStr">
         <is>
           <t>TC-6408b44286</t>
         </is>
       </c>
-      <c r="F151" s="3" t="inlineStr">
+      <c r="F150" s="3" t="inlineStr">
         <is>
           <t>Prove D4 refuses to let the respondent past when it is left blank. The questionnaire marks it compulsory, and it is a single question</t>
         </is>
       </c>
-      <c r="G151" s="3" t="inlineStr">
+      <c r="G150" s="3" t="inlineStr">
         <is>
           <t>1. S1 = Yes
 2. S2 = Personally manage an ongoing chronic health condition
@@ -11294,58 +11218,58 @@
 26. D3 = Woman</t>
         </is>
       </c>
-      <c r="H151" s="3" t="inlineStr">
+      <c r="H150" s="3" t="inlineStr">
         <is>
           <t>At D4, select nothing at all, then submit.</t>
         </is>
       </c>
-      <c r="I151" s="3" t="inlineStr">
+      <c r="I150" s="3" t="inlineStr">
         <is>
           <t>1. the survey REFUSES to move on; the same page reappears
 2. an error message is shown against D4</t>
         </is>
       </c>
-      <c r="J151" s="2" t="inlineStr">
+      <c r="J150" s="2" t="inlineStr">
         <is>
           <t>Blank answer is blocked</t>
         </is>
       </c>
-      <c r="K151" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" s="2" t="n">
-        <v>151</v>
-      </c>
-      <c r="B152" s="2" t="inlineStr">
+      <c r="K150" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="B151" s="2" t="inlineStr">
         <is>
           <t>Q22</t>
         </is>
       </c>
-      <c r="C152" s="3" t="inlineStr">
+      <c r="C151" s="3" t="inlineStr">
         <is>
           <t>Q22 | May we use your anonymized comments in internal reporting? | single | Yes; No | Always show</t>
         </is>
       </c>
-      <c r="D152" s="2" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="E152" s="2" t="inlineStr">
+      <c r="D151" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E151" s="2" t="inlineStr">
         <is>
           <t>TC-d3a3106833</t>
         </is>
       </c>
-      <c r="F152" s="3" t="inlineStr">
+      <c r="F151" s="3" t="inlineStr">
         <is>
           <t>Prove the survey flows correctly at Q22: answer it normally and the respondent should move on to whatever the questionnaire says comes next, not stop or jump elsewhere</t>
         </is>
       </c>
-      <c r="G152" s="3" t="inlineStr">
+      <c r="G151" s="3" t="inlineStr">
         <is>
           <t>1. S1 = Yes
 2. S2 = Personally manage an ongoing chronic health condition
@@ -11377,58 +11301,58 @@
 28. Q22 = Yes</t>
         </is>
       </c>
-      <c r="H152" s="3" t="inlineStr">
+      <c r="H151" s="3" t="inlineStr">
         <is>
           <t>Answer through the whole survey as listed, then observe where it ends.</t>
         </is>
       </c>
-      <c r="I152" s="3" t="inlineStr">
+      <c r="I151" s="3" t="inlineStr">
         <is>
           <t>1. Q22 IS shown on the page
 2. the next question shown is Q23</t>
         </is>
       </c>
-      <c r="J152" s="2" t="inlineStr">
+      <c r="J151" s="2" t="inlineStr">
         <is>
           <t>Shows / hides correctly</t>
         </is>
       </c>
-      <c r="K152" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" s="2" t="n">
-        <v>152</v>
-      </c>
-      <c r="B153" s="2" t="inlineStr">
+      <c r="K151" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="n">
+        <v>151</v>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
         <is>
           <t>Q22</t>
         </is>
       </c>
-      <c r="C153" s="3" t="inlineStr">
+      <c r="C152" s="3" t="inlineStr">
         <is>
           <t>Q22 | May we use your anonymized comments in internal reporting? | single | Yes; No | Always show</t>
         </is>
       </c>
-      <c r="D153" s="2" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="E153" s="2" t="inlineStr">
+      <c r="D152" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E152" s="2" t="inlineStr">
         <is>
           <t>TC-7596aff04a</t>
         </is>
       </c>
-      <c r="F153" s="3" t="inlineStr">
+      <c r="F152" s="3" t="inlineStr">
         <is>
           <t>Prove Q22 refuses to let the respondent past when it is left blank. The questionnaire marks it compulsory, and it is a single question</t>
         </is>
       </c>
-      <c r="G153" s="3" t="inlineStr">
+      <c r="G152" s="3" t="inlineStr">
         <is>
           <t>1. S1 = Yes
 2. S2 = Personally manage an ongoing chronic health condition
@@ -11459,59 +11383,59 @@
 27. D4 = Band 1</t>
         </is>
       </c>
-      <c r="H153" s="3" t="inlineStr">
+      <c r="H152" s="3" t="inlineStr">
         <is>
           <t>At Q22, select nothing at all, then submit.</t>
         </is>
       </c>
-      <c r="I153" s="3" t="inlineStr">
+      <c r="I152" s="3" t="inlineStr">
         <is>
           <t>1. the survey REFUSES to move on; the same page reappears
 2. an error message is shown against Q22</t>
         </is>
       </c>
-      <c r="J153" s="2" t="inlineStr">
+      <c r="J152" s="2" t="inlineStr">
         <is>
           <t>Blank answer is blocked</t>
         </is>
       </c>
-      <c r="K153" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" s="2" t="n">
-        <v>153</v>
-      </c>
-      <c r="B154" s="2" t="inlineStr">
+      <c r="K152" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="n">
+        <v>152</v>
+      </c>
+      <c r="B153" s="2" t="inlineStr">
         <is>
           <t>Q23</t>
         </is>
       </c>
-      <c r="C154" s="3" t="inlineStr">
+      <c r="C153" s="3" t="inlineStr">
         <is>
           <t>Q23 | Any final comments? | text | — | Validate: {"max_length": 1000}
 Optional</t>
         </is>
       </c>
-      <c r="D154" s="2" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="E154" s="2" t="inlineStr">
+      <c r="D153" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E153" s="2" t="inlineStr">
         <is>
           <t>TC-66de0d40bf</t>
         </is>
       </c>
-      <c r="F154" s="3" t="inlineStr">
+      <c r="F153" s="3" t="inlineStr">
         <is>
           <t>Prove the survey flows correctly at Q23: answer it normally and the respondent should move on to whatever the questionnaire says comes next, not stop or jump elsewhere</t>
         </is>
       </c>
-      <c r="G154" s="3" t="inlineStr">
+      <c r="G153" s="3" t="inlineStr">
         <is>
           <t>1. S1 = Yes
 2. S2 = Personally manage an ongoing chronic health condition
@@ -11543,59 +11467,59 @@
 28. Q22 = Yes</t>
         </is>
       </c>
-      <c r="H154" s="3" t="inlineStr">
+      <c r="H153" s="3" t="inlineStr">
         <is>
           <t>Answer through the whole survey as listed, then observe where it ends.</t>
         </is>
       </c>
-      <c r="I154" s="3" t="inlineStr">
+      <c r="I153" s="3" t="inlineStr">
         <is>
           <t>1. Q23 IS shown on the page
 2. the respondent reaches the normal thank-you page</t>
         </is>
       </c>
-      <c r="J154" s="2" t="inlineStr">
+      <c r="J153" s="2" t="inlineStr">
         <is>
           <t>Shows / hides correctly</t>
         </is>
       </c>
-      <c r="K154" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" s="2" t="n">
-        <v>154</v>
-      </c>
-      <c r="B155" s="2" t="inlineStr">
+      <c r="K153" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="n">
+        <v>153</v>
+      </c>
+      <c r="B154" s="2" t="inlineStr">
         <is>
           <t>Q23</t>
         </is>
       </c>
-      <c r="C155" s="3" t="inlineStr">
+      <c r="C154" s="3" t="inlineStr">
         <is>
           <t>Q23 | Any final comments? | text | — | Validate: {"max_length": 1000}
 Optional</t>
         </is>
       </c>
-      <c r="D155" s="2" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="E155" s="2" t="inlineStr">
+      <c r="D154" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E154" s="2" t="inlineStr">
         <is>
           <t>TC-27239f8502</t>
         </is>
       </c>
-      <c r="F155" s="3" t="inlineStr">
+      <c r="F154" s="3" t="inlineStr">
         <is>
           <t>Prove Q23 ACCEPTS an answer that obeys its rule. The QRE's rule is: the answer must be at most 1000 characters</t>
         </is>
       </c>
-      <c r="G155" s="3" t="inlineStr">
+      <c r="G154" s="3" t="inlineStr">
         <is>
           <t>1. S1 = Yes
 2. S2 = Personally manage an ongoing chronic health condition
@@ -11627,58 +11551,58 @@
 28. Q22 = Yes</t>
         </is>
       </c>
-      <c r="H155" s="3" t="inlineStr">
+      <c r="H154" s="3" t="inlineStr">
         <is>
           <t>At Q23, type “x”, then submit.</t>
         </is>
       </c>
-      <c r="I155" s="3" t="inlineStr">
+      <c r="I154" s="3" t="inlineStr">
         <is>
           <t>1. the survey ACCEPTS the answer and moves to the next page</t>
         </is>
       </c>
-      <c r="J155" s="2" t="inlineStr">
+      <c r="J154" s="2" t="inlineStr">
         <is>
           <t>Answer rule accepts or rejects</t>
         </is>
       </c>
-      <c r="K155" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" s="2" t="n">
-        <v>155</v>
-      </c>
-      <c r="B156" s="2" t="inlineStr">
+      <c r="K154" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="n">
+        <v>154</v>
+      </c>
+      <c r="B155" s="2" t="inlineStr">
         <is>
           <t>Q23</t>
         </is>
       </c>
-      <c r="C156" s="3" t="inlineStr">
+      <c r="C155" s="3" t="inlineStr">
         <is>
           <t>Q23 | Any final comments? | text | — | Validate: {"max_length": 1000}
 Optional</t>
         </is>
       </c>
-      <c r="D156" s="2" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="E156" s="2" t="inlineStr">
+      <c r="D155" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E155" s="2" t="inlineStr">
         <is>
           <t>TC-de6bfa278d</t>
         </is>
       </c>
-      <c r="F156" s="3" t="inlineStr">
+      <c r="F155" s="3" t="inlineStr">
         <is>
           <t>Prove Q23 REJECTS an answer that breaks its rule. The QRE's rule is: the answer must be at most 1000 characters</t>
         </is>
       </c>
-      <c r="G156" s="3" t="inlineStr">
+      <c r="G155" s="3" t="inlineStr">
         <is>
           <t>1. S1 = Yes
 2. S2 = Personally manage an ongoing chronic health condition
@@ -11710,59 +11634,59 @@
 28. Q22 = Yes</t>
         </is>
       </c>
-      <c r="H156" s="3" t="inlineStr">
+      <c r="H155" s="3" t="inlineStr">
         <is>
           <t>At Q23, type a 1001-character answer, then submit.</t>
         </is>
       </c>
-      <c r="I156" s="3" t="inlineStr">
+      <c r="I155" s="3" t="inlineStr">
         <is>
           <t>1. the survey REFUSES to move on; the same page reappears
 2. an error message is shown against Q23</t>
         </is>
       </c>
-      <c r="J156" s="2" t="inlineStr">
+      <c r="J155" s="2" t="inlineStr">
         <is>
           <t>Answer rule accepts or rejects</t>
         </is>
       </c>
-      <c r="K156" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" s="2" t="n">
-        <v>156</v>
-      </c>
-      <c r="B157" s="2" t="inlineStr">
+      <c r="K155" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="n">
+        <v>155</v>
+      </c>
+      <c r="B156" s="2" t="inlineStr">
         <is>
           <t>Q23</t>
         </is>
       </c>
-      <c r="C157" s="3" t="inlineStr">
+      <c r="C156" s="3" t="inlineStr">
         <is>
           <t>Q23 | Any final comments? | text | — | Validate: {"max_length": 1000}
 Optional</t>
         </is>
       </c>
-      <c r="D157" s="2" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="E157" s="2" t="inlineStr">
+      <c r="D156" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E156" s="2" t="inlineStr">
         <is>
           <t>TC-501913f6da</t>
         </is>
       </c>
-      <c r="F157" s="3" t="inlineStr">
+      <c r="F156" s="3" t="inlineStr">
         <is>
           <t>Prove Q23 lets the respondent through with no answer, because the questionnaire marks it optional</t>
         </is>
       </c>
-      <c r="G157" s="3" t="inlineStr">
+      <c r="G156" s="3" t="inlineStr">
         <is>
           <t>1. S1 = Yes
 2. S2 = Personally manage an ongoing chronic health condition
@@ -11794,58 +11718,58 @@
 28. Q22 = Yes</t>
         </is>
       </c>
-      <c r="H157" s="3" t="inlineStr">
+      <c r="H156" s="3" t="inlineStr">
         <is>
           <t>At Q23, type nothing, then submit.</t>
         </is>
       </c>
-      <c r="I157" s="3" t="inlineStr">
+      <c r="I156" s="3" t="inlineStr">
         <is>
           <t>1. the survey ACCEPTS the answer and moves to the next page</t>
         </is>
       </c>
-      <c r="J157" s="2" t="inlineStr">
+      <c r="J156" s="2" t="inlineStr">
         <is>
           <t>Blank answer is blocked</t>
         </is>
       </c>
-      <c r="K157" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="158">
-      <c r="A158" s="2" t="n">
-        <v>157</v>
-      </c>
-      <c r="B158" s="2" t="inlineStr">
+      <c r="K156" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="2" t="n">
+        <v>156</v>
+      </c>
+      <c r="B157" s="2" t="inlineStr">
         <is>
           <t>Q23</t>
         </is>
       </c>
-      <c r="C158" s="3" t="inlineStr">
+      <c r="C157" s="3" t="inlineStr">
         <is>
           <t>Q23 | Any final comments? | text | — | Validate: {"max_length": 1000}
 Optional</t>
         </is>
       </c>
-      <c r="D158" s="2" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="E158" s="2" t="inlineStr">
+      <c r="D157" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E157" s="2" t="inlineStr">
         <is>
           <t>TC-e8a2b0563a</t>
         </is>
       </c>
-      <c r="F158" s="3" t="inlineStr">
+      <c r="F157" s="3" t="inlineStr">
         <is>
           <t>Prove Q23 REJECTS an answer that breaks its rule. The QRE's rule is: the answer must be at most 1000 characters</t>
         </is>
       </c>
-      <c r="G158" s="3" t="inlineStr">
+      <c r="G157" s="3" t="inlineStr">
         <is>
           <t>1. S1 = Yes
 2. S2 = Personally manage an ongoing chronic health condition
@@ -11877,58 +11801,58 @@
 28. Q22 = Yes</t>
         </is>
       </c>
-      <c r="H158" s="3" t="inlineStr">
+      <c r="H157" s="3" t="inlineStr">
         <is>
           <t>At Q23, type a 1000-character answer, then submit.</t>
         </is>
       </c>
-      <c r="I158" s="3" t="inlineStr">
+      <c r="I157" s="3" t="inlineStr">
         <is>
           <t>1. the survey ACCEPTS the answer and moves to the next page</t>
         </is>
       </c>
-      <c r="J158" s="2" t="inlineStr">
+      <c r="J157" s="2" t="inlineStr">
         <is>
           <t>Answer rule accepts or rejects</t>
         </is>
       </c>
-      <c r="K158" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" s="2" t="n">
-        <v>158</v>
-      </c>
-      <c r="B159" s="2" t="inlineStr">
+      <c r="K157" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="n">
+        <v>157</v>
+      </c>
+      <c r="B158" s="2" t="inlineStr">
         <is>
           <t>Q23</t>
         </is>
       </c>
-      <c r="C159" s="3" t="inlineStr">
+      <c r="C158" s="3" t="inlineStr">
         <is>
           <t>Q23 | Any final comments? | text | — | Validate: {"max_length": 1000}
 Optional</t>
         </is>
       </c>
-      <c r="D159" s="2" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="E159" s="2" t="inlineStr">
+      <c r="D158" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E158" s="2" t="inlineStr">
         <is>
           <t>TC-40e56a8b6b</t>
         </is>
       </c>
-      <c r="F159" s="3" t="inlineStr">
+      <c r="F158" s="3" t="inlineStr">
         <is>
           <t>Prove Q23 REJECTS an answer that breaks its rule. The QRE's rule is: the answer must be at most 1000 characters</t>
         </is>
       </c>
-      <c r="G159" s="3" t="inlineStr">
+      <c r="G158" s="3" t="inlineStr">
         <is>
           <t>1. S1 = Yes
 2. S2 = Personally manage an ongoing chronic health condition
@@ -11960,58 +11884,58 @@
 28. Q22 = Yes</t>
         </is>
       </c>
-      <c r="H159" s="3" t="inlineStr">
+      <c r="H158" s="3" t="inlineStr">
         <is>
           <t>At Q23, type “O'Brien said "yes" &lt;50% &amp; more”, then submit.</t>
         </is>
       </c>
-      <c r="I159" s="3" t="inlineStr">
+      <c r="I158" s="3" t="inlineStr">
         <is>
           <t>1. the survey ACCEPTS the answer and moves to the next page</t>
         </is>
       </c>
-      <c r="J159" s="2" t="inlineStr">
+      <c r="J158" s="2" t="inlineStr">
         <is>
           <t>Answer rule accepts or rejects</t>
         </is>
       </c>
-      <c r="K159" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" s="2" t="n">
-        <v>159</v>
-      </c>
-      <c r="B160" s="2" t="inlineStr">
+      <c r="K158" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="2" t="n">
+        <v>158</v>
+      </c>
+      <c r="B159" s="2" t="inlineStr">
         <is>
           <t>Q23</t>
         </is>
       </c>
-      <c r="C160" s="3" t="inlineStr">
+      <c r="C159" s="3" t="inlineStr">
         <is>
           <t>Q23 | Any final comments? | text | — | Validate: {"max_length": 1000}
 Optional</t>
         </is>
       </c>
-      <c r="D160" s="2" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="E160" s="2" t="inlineStr">
+      <c r="D159" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E159" s="2" t="inlineStr">
         <is>
           <t>TC-38d0f2db08</t>
         </is>
       </c>
-      <c r="F160" s="3" t="inlineStr">
+      <c r="F159" s="3" t="inlineStr">
         <is>
           <t>Prove Q23 refuses to let the respondent past when it is left blank. The questionnaire marks it compulsory, and it is a text question</t>
         </is>
       </c>
-      <c r="G160" s="3" t="inlineStr">
+      <c r="G159" s="3" t="inlineStr">
         <is>
           <t>1. S1 = Yes
 2. S2 = Personally manage an ongoing chronic health condition
@@ -12043,53 +11967,53 @@
 28. Q22 = Yes</t>
         </is>
       </c>
-      <c r="H160" s="3" t="inlineStr">
+      <c r="H159" s="3" t="inlineStr">
         <is>
           <t>At Q23, type 3 spaces and nothing else, then submit.</t>
         </is>
       </c>
-      <c r="I160" s="3" t="inlineStr">
+      <c r="I159" s="3" t="inlineStr">
         <is>
           <t>1. the survey ACCEPTS the answer and moves to the next page</t>
         </is>
       </c>
-      <c r="J160" s="2" t="inlineStr">
+      <c r="J159" s="2" t="inlineStr">
         <is>
           <t>Blank answer is blocked</t>
         </is>
       </c>
-      <c r="K160" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" s="2" t="n">
-        <v>160</v>
-      </c>
-      <c r="B161" s="2" t="inlineStr">
+      <c r="K159" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="n">
+        <v>159</v>
+      </c>
+      <c r="B160" s="2" t="inlineStr">
         <is>
           <t>whole survey</t>
         </is>
       </c>
-      <c r="C161" s="3" t="inlineStr"/>
-      <c r="D161" s="2" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="E161" s="2" t="inlineStr">
+      <c r="C160" s="3" t="inlineStr"/>
+      <c r="D160" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E160" s="2" t="inlineStr">
         <is>
           <t>TC-236280087d</t>
         </is>
       </c>
-      <c r="F161" s="3" t="inlineStr">
+      <c r="F160" s="3" t="inlineStr">
         <is>
           <t>Prove the survey finishes normally for a respondent who answers everything and triggers no screen-out</t>
         </is>
       </c>
-      <c r="G161" s="3" t="inlineStr">
+      <c r="G160" s="3" t="inlineStr">
         <is>
           <t>1. S1 = Yes
 2. S2 = Personally manage an ongoing chronic health condition
@@ -12121,22 +12045,22 @@
 28. Q22 = Yes</t>
         </is>
       </c>
-      <c r="H161" s="3" t="inlineStr">
+      <c r="H160" s="3" t="inlineStr">
         <is>
           <t>Answer through the whole survey as listed, then observe where it ends.</t>
         </is>
       </c>
-      <c r="I161" s="3" t="inlineStr">
+      <c r="I160" s="3" t="inlineStr">
         <is>
           <t>1. the respondent reaches the normal thank-you page</t>
         </is>
       </c>
-      <c r="J161" s="2" t="inlineStr">
+      <c r="J160" s="2" t="inlineStr">
         <is>
           <t>Survey ends in the right place</t>
         </is>
       </c>
-      <c r="K161" s="2" t="inlineStr">
+      <c r="K160" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>

</xml_diff>